<commit_message>
Updated FIN model - 2025-09-13 09:10
</commit_message>
<xml_diff>
--- a/VerveStacks_FIN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_FIN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FIN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{439DBB46-C8B9-420C-9B60-8C73F7EB673F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2935784-9539-4BC0-9A20-2AC3DFA4A314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6324,7 +6324,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B93A189F-AD77-40AD-8595-DD4DB2E9DFA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42CF19EE-BD11-451B-B59C-3CBB7273DB2F}">
   <dimension ref="B9:N11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6418,7 +6418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62E4CFC-A609-4138-B777-B2BC314789DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501FF7EB-6DA5-4552-AEEB-DA34FDF01586}">
   <dimension ref="B9:AB86"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10736,7 +10736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC97DD9-02AD-4AF1-BB12-ABCF88077D5C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{291DA346-B084-494F-8B5B-9B9AFC7B0652}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FIN model - 2025-09-13 09:52
</commit_message>
<xml_diff>
--- a/VerveStacks_FIN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_FIN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FIN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2935784-9539-4BC0-9A20-2AC3DFA4A314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{473B885E-9E87-42CB-BFCE-FDABE3EE0E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6324,7 +6324,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42CF19EE-BD11-451B-B59C-3CBB7273DB2F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B325784B-B2FB-4F58-8BE5-008893C4DC5B}">
   <dimension ref="B9:N11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6418,7 +6418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501FF7EB-6DA5-4552-AEEB-DA34FDF01586}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35192DAE-1695-43A0-863C-0791DA84DCCF}">
   <dimension ref="B9:AB86"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10736,7 +10736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{291DA346-B084-494F-8B5B-9B9AFC7B0652}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94EE74CE-D5D8-48D2-B4E6-FA3F1FBEF0C8}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>